<commit_message>
Redemption module TestCases Update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/06_RewardCatalogue/RewardCatalogue/02_RedemptionCartPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/06_RewardCatalogue/RewardCatalogue/02_RedemptionCartPageTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\06_RewardCatalogue\RewardCatalogue\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9F5059-F9AE-46D4-A611-28765F34A74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F819ED1-C220-47E2-ABDD-E1858C3B3693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="80">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -365,6 +365,9 @@
     <t>waitforsnackbardisappear
 redemptioncart_clickon_cancelbtn
 verifypagetitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -1310,7 +1313,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{089D5808-B2AF-4105-BEF8-05FAA4CBE122}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1768,7 +1771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1795,6 +1798,9 @@
       </c>
       <c r="K17" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>